<commit_message>
Stories added upto 6
</commit_message>
<xml_diff>
--- a/NRM1_Cost_Estimate_Tool_v4_5.xlsx
+++ b/NRM1_Cost_Estimate_Tool_v4_5.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\nabil\estates-ai-tool\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8FBA7215-3F23-4322-836E-C3ED81F6A740}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7A8CB13B-2BB0-4BE9-9D19-89039DCA18AD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -3082,7 +3082,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="5" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A5" s="56" t="s">
         <v>21</v>
       </c>
@@ -3105,7 +3105,7 @@
       <c r="R5" s="57"/>
       <c r="S5" s="58"/>
     </row>
-    <row r="6" spans="1:19" ht="25.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:19" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A6" s="47" t="s">
         <v>22</v>
       </c>
@@ -3164,7 +3164,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="7" spans="1:19" ht="25.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:19" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A7" s="50" t="s">
         <v>30</v>
       </c>
@@ -3223,7 +3223,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="8" spans="1:19" ht="25.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:19" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A8" s="47" t="s">
         <v>34</v>
       </c>
@@ -3282,7 +3282,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="9" spans="1:19" ht="25.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:19" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A9" s="50" t="s">
         <v>37</v>
       </c>
@@ -3341,7 +3341,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="10" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A10" s="56" t="s">
         <v>40</v>
       </c>
@@ -3364,7 +3364,7 @@
       <c r="R10" s="57"/>
       <c r="S10" s="58"/>
     </row>
-    <row r="11" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A11" s="47" t="s">
         <v>41</v>
       </c>
@@ -3423,7 +3423,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="12" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A12" s="50" t="s">
         <v>44</v>
       </c>
@@ -3482,7 +3482,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="13" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A13" s="47" t="s">
         <v>47</v>
       </c>
@@ -3541,7 +3541,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="14" spans="1:19" ht="25.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:19" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A14" s="50" t="s">
         <v>50</v>
       </c>
@@ -3600,7 +3600,7 @@
         <v>658</v>
       </c>
     </row>
-    <row r="15" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A15" s="56" t="s">
         <v>52</v>
       </c>
@@ -3623,7 +3623,7 @@
       <c r="R15" s="57"/>
       <c r="S15" s="58"/>
     </row>
-    <row r="16" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A16" s="47" t="s">
         <v>53</v>
       </c>
@@ -3682,7 +3682,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="17" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A17" s="50" t="s">
         <v>56</v>
       </c>
@@ -3741,7 +3741,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="18" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A18" s="47" t="s">
         <v>59</v>
       </c>
@@ -3800,7 +3800,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="19" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A19" s="50" t="s">
         <v>62</v>
       </c>
@@ -3859,7 +3859,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="20" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A20" s="47" t="s">
         <v>65</v>
       </c>
@@ -3918,7 +3918,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="21" spans="1:19" ht="25.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:19" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A21" s="50" t="s">
         <v>68</v>
       </c>
@@ -3977,7 +3977,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="22" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A22" s="47" t="s">
         <v>71</v>
       </c>
@@ -4036,7 +4036,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="23" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A23" s="50" t="s">
         <v>74</v>
       </c>
@@ -4095,7 +4095,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="24" spans="1:19" ht="25.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:19" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A24" s="47" t="s">
         <v>77</v>
       </c>
@@ -4212,19 +4212,19 @@
         <v>55</v>
       </c>
       <c r="L26" s="49">
-        <v>180</v>
+        <v>140</v>
       </c>
       <c r="M26" s="49">
         <v>55</v>
       </c>
       <c r="N26" s="49">
-        <v>180</v>
+        <v>140</v>
       </c>
       <c r="O26" s="49">
         <v>55</v>
       </c>
       <c r="P26" s="49">
-        <v>140</v>
+        <v>120</v>
       </c>
       <c r="Q26" s="49">
         <v>0</v>
@@ -4271,19 +4271,19 @@
         <v>75</v>
       </c>
       <c r="L27" s="53">
-        <v>280</v>
+        <v>200</v>
       </c>
       <c r="M27" s="53">
         <v>75</v>
       </c>
       <c r="N27" s="53">
-        <v>280</v>
+        <v>200</v>
       </c>
       <c r="O27" s="53">
         <v>80</v>
       </c>
       <c r="P27" s="53">
-        <v>200</v>
+        <v>140</v>
       </c>
       <c r="Q27" s="53">
         <v>0</v>
@@ -6475,16 +6475,16 @@
         <v>90</v>
       </c>
       <c r="M68" s="49">
-        <v>45</v>
+        <v>50</v>
       </c>
       <c r="N68" s="49">
-        <v>70</v>
+        <v>90</v>
       </c>
       <c r="O68" s="49">
-        <v>30</v>
+        <v>50</v>
       </c>
       <c r="P68" s="49">
-        <v>65</v>
+        <v>90</v>
       </c>
       <c r="Q68" s="49">
         <v>0</v>
@@ -6646,10 +6646,10 @@
         <v>30</v>
       </c>
       <c r="K71" s="53">
-        <v>55</v>
+        <v>90</v>
       </c>
       <c r="L71" s="53">
-        <v>200</v>
+        <v>180</v>
       </c>
       <c r="M71" s="53">
         <v>150</v>

</xml_diff>